<commit_message>
trying to figure out SQL vs. friendly script for both column and filter
</commit_message>
<xml_diff>
--- a/output/Campus FY 2025-26 annual statistics NZ-level report/2025 - 2026/exclusions tab/UCB_targeted_review_FY2025-26_exclusions_documentation_as_of_2026-07-09.xlsx
+++ b/output/Campus FY 2025-26 annual statistics NZ-level report/2025 - 2026/exclusions tab/UCB_targeted_review_FY2025-26_exclusions_documentation_as_of_2026-07-09.xlsx
@@ -3634,7 +3634,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="55">
       <c r="A55" s="32" t="inlineStr">
         <is>
-          <t>"Portfolio Library Unit"."Library Name" is equal to / is in X_Do_Not_Use_</t>
+          <t>"Portfolio Library Unit"."Library Name" LIKE 'X_Do_Not_Use_%'</t>
         </is>
       </c>
       <c r="B55" s="39" t="inlineStr">
@@ -5711,7 +5711,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="86">
       <c r="A86" s="32" t="inlineStr">
         <is>
-          <t>"Electronic Collection"."Electronic Collection Public Name" is equal to / is in Ebook Central Perpetual, DDA and Subscription Titles; EBSCO (UCSD). eBook Collection DDA online monographs.; R2 Digital Library DDA</t>
+          <t>"Electronic Collection"."Electronic Collection Public Name" IN ('Ebook Central Perpetual, DDA and Subscription Titles', 'EBSCO (UCSD). eBook Collection DDA online monographs.', 'R2 Digital Library DDA')</t>
         </is>
       </c>
       <c r="B86" s="39" t="inlineStr">
@@ -5778,7 +5778,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="87">
       <c r="A87" s="32" t="inlineStr">
         <is>
-          <t>"Electronic Collection"."Electronic Collection Public Name" is equal to / is in British and Irish Women's Letters and Diaries: First Edition (Pre-January 2009 Purchasers Only); Books@Ovid - LWW JBIB Book Collection 2017-2018 Purchase; Books@Ovid Purchase; Books@Ovid Purchase Complete; North American Indian Drama: First Edition (Pre-October 2012 Purchasers Only); Twentieth Century North American Drama: First Edition (Pre-October 2012 Purchasers Only); Institute of Physics Historic Archive Purchase; Maruzen eBook Library; Berkeley LDC purchases; IGI Global Evidence Based PURCHASED; Oxford University Press Anthropology Local Purchased Collection; Sage EBS; Sage online monographs EBS (Sage EBS) purchased; UC Davis locally purchased monographs_LOCAL; UCSC owned streaming video; African Writers Series (pre-September 2011 purchase); SAGE Complete Deep Backfile Purchase 2008; SAGE Deep Backfile Upgrade Purchase 2009; SAGE Deep Backfile Upgrade Purchase 2010; SAGE Deep Backfile Upgrade Purchase 2011; SAGE Deep Backfile Upgrade Purchase 2012; SAGE Deep Backfile Upgrade Purchase 2013; SAGE Deep Backfile Upgrade Purchase 2014; SAGE Deep Backfile Upgrade Purchase 2015; SAGE Deep Backfile Upgrade Purchase 2016; SAGE Deep Backfile Upgrade Purchase 2017; SAGE Psychology Subject Collection Backfile Purchase; Taylor &amp; Francis online monographs (EBS) purchased</t>
+          <t>"Electronic Collection"."Electronic Collection Public Name" IN ('British and Irish Women''s Letters and Diaries: First Edition (Pre-January 2009 Purchasers Only)', 'Books@Ovid - LWW JBIB Book Collection 2017-2018 Purchase', 'Books@Ovid Purchase', 'Books@Ovid Purchase Complete', 'North American Indian Drama: First Edition (Pre-October 2012 Purchasers Only)', 'Twentieth Century North American Drama: First Edition (Pre-October 2012 Purchasers Only)', 'Institute of Physics Historic Archive Purchase', 'Maruzen eBook Library', 'Berkeley LDC purchases', 'IGI Global Evidence Based PURCHASED', 'Oxford University Press Anthropology Local Purchased Collection', 'Sage EBS', 'Sage online monographs EBS (Sage EBS) purchased', 'UC Davis locally purchased monographs_LOCAL', 'UCSC owned streaming video', 'African Writers Series (pre-September 2011 purchase)', 'SAGE Complete Deep Backfile Purchase 2008', 'SAGE Deep Backfile Upgrade Purchase 2009', 'SAGE Deep Backfile Upgrade Purchase 2010', 'SAGE Deep Backfile Upgrade Purchase 2011', 'SAGE Deep Backfile Upgrade Purchase 2012', 'SAGE Deep Backfile Upgrade Purchase 2013', 'SAGE Deep Backfile Upgrade Purchase 2014', 'SAGE Deep Backfile Upgrade Purchase 2015', 'SAGE Deep Backfile Upgrade Purchase 2016', 'SAGE Deep Backfile Upgrade Purchase 2017', 'SAGE Psychology Subject Collection Backfile Purchase', 'Taylor &amp; Francis online monographs (EBS) purchased')</t>
         </is>
       </c>
       <c r="B87" s="39" t="inlineStr">
@@ -5845,7 +5845,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="88">
       <c r="A88" s="32" t="inlineStr">
         <is>
-          <t>"Electronic Collection"."Electronic Collection Public Name"</t>
+          <t>"Electronic Collection"."Electronic Collection Public Name" IS NULL</t>
         </is>
       </c>
       <c r="B88" s="39" t="inlineStr">
@@ -6448,7 +6448,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="97">
       <c r="A97" s="32" t="inlineStr">
         <is>
-          <t>"Institution"."Institution Name"6532</t>
+          <t>"Institution"."Institution Name" = 6532</t>
         </is>
       </c>
       <c r="B97" s="39" t="inlineStr">
@@ -11071,7 +11071,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="166">
       <c r="A166" s="32" t="inlineStr">
         <is>
-          <t>"Item Location at Time of Loan"."Location Code" is equal to / is in UNASSIGNED; ah92; ah9e; drr; zs; ea9r; qc9m; qn9c; muv; esx</t>
+          <t>"Item Location at Time of Loan"."Location Code" IN ('UNASSIGNED', 'ah92', 'ah9e', 'drr', 'zs', 'ea9r', 'qc9m', 'qn9c', 'muv', 'esx')</t>
         </is>
       </c>
       <c r="B166" s="39" t="inlineStr">
@@ -11138,7 +11138,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="167">
       <c r="A167" s="32" t="inlineStr">
         <is>
-          <t>"Item Location at Time of Loan"."Location Code" is equal to / is in bu; chs; ma9f; ma9e; ev9t; gs; mts; mf9f; mf9e; mf; mfs; so9f; so9e</t>
+          <t>"Item Location at Time of Loan"."Location Code" IN ('bu', 'chs', 'ma9f', 'ma9e', 'ev9t', 'gs', 'mts', 'mf9f', 'mf9e', 'mf', 'mfs', 'so9f', 'so9e')</t>
         </is>
       </c>
       <c r="B167" s="39" t="inlineStr">
@@ -11272,7 +11272,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="169">
       <c r="A169" s="32" t="inlineStr">
         <is>
-          <t>"Item Location at Time of Loan"."Location Code" is equal to / is in OUT_RS_REQ; IN_RS_REQ</t>
+          <t>"Item Location at Time of Loan"."Location Code" IN ('OUT_RS_REQ', 'IN_RS_REQ')</t>
         </is>
       </c>
       <c r="B169" s="39" t="inlineStr">
@@ -11339,7 +11339,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="170">
       <c r="A170" s="32" t="inlineStr">
         <is>
-          <t>"Item Location at Time of Loan"."Location Code" is equal to / is in an; ah; ah9t; ahu; ah9a; ah9l; ah9d; ah95; ah9g; ah9j; tb; tb2; tbo; tb9u; tb9o; tb9p; tb95; tb94; tbr; tbw; tbv; tp; tu; tuo; tu94; bi; bic; bi9c; bif; bil; bim; bi9b; binb; bik; bir; bis; bi9d; buc; bus; ch; chc; chnb; chp; chr; dr; ma; mac; ucbears; zw; es; es93; es9c; esi; es9m; es9b; es9d; ess; esw; ea; eao; eat; eau; eav; ear; eas; eax; ea9w; en; en9c; enc; en9i; ens; ensp; ev; evr; evp; ev2; evpo; evo; evu; evs; qa; qc; qcl; qe; qe9f; qn; qn9k; qn9m; ig; igr; igs; it; ite; iti; ith; itp; its; lb; lb9l; mt; mtp; mta; mc; mo; mo9a; mo9f; moga; mo9g; mo9m; mo9n; mo9p; mo9y; mo9s; mo9t; mu; mu9m; mu9x; muc; mu9c; muo; mu9f; dn; nbqar; nbtbr; nbtnr; nntnr; nbqcr; nbqer; nbear; nbevr; nbcer; nbitr; nbmar; nbmnr; nbmcr; nbmur; nbqnr; nncl; npupr; nban; nbah; nbbi; nbbu; nbch; nbes; nbea; nben; nbev; nbig; nbit; nblw; nbma; nbmt; nbmu; nbdn; nbph; nbso; nbss; nddo; ndhe; ndla; ndph; ndsh; nlxx; nrxx; nsxx; ncmh; ncme; ncsc; nfge; nucl; nu03u; nuht; nu01u; nu02u; nu03b; nu01b; nu02b; nbphr; nbtur; ndspr; nlyrr; ncspr; nfspr; php; phs; so; sos; esnb; es97; eanb; eaob; ennb; nbbir; nbchr; nbdnr; ndag</t>
+          <t>"Item Location at Time of Loan"."Location Code" IN ('an', 'ah', 'ah9t', 'ahu', 'ah9a', 'ah9l', 'ah9d', 'ah95', 'ah9g', 'ah9j', 'tb', 'tb2', 'tbo', 'tb9u', 'tb9o', 'tb9p', 'tb95', 'tb94', 'tbr', 'tbw', 'tbv', 'tp', 'tu', 'tuo', 'tu94', 'bi', 'bic', 'bi9c', 'bif', 'bil', 'bim', 'bi9b', 'binb', 'bik', 'bir', 'bis', 'bi9d', 'buc', 'bus', 'ch', 'chc', 'chnb', 'chp', 'chr', 'dr', 'ma', 'mac', 'ucbears', 'zw', 'es', 'es93', 'es9c', 'esi', 'es9m', 'es9b', 'es9d', 'ess', 'esw', 'ea', 'eao', 'eat', 'eau', 'eav', 'ear', 'eas', 'eax', 'ea9w', 'en', 'en9c', 'enc', 'en9i', 'ens', 'ensp', 'ev', 'evr', 'evp', 'ev2', 'evpo', 'evo', 'evu', 'evs', 'qa', 'qc', 'qcl', 'qe', 'qe9f', 'qn', 'qn9k', 'qn9m', 'ig', 'igr', 'igs', 'it', 'ite', 'iti', 'ith', 'itp', 'its', 'lb', 'lb9l', 'mt', 'mtp', 'mta', 'mc', 'mo', 'mo9a', 'mo9f', 'moga', 'mo9g', 'mo9m', 'mo9n', 'mo9p', 'mo9y', 'mo9s', 'mo9t', 'mu', 'mu9m', 'mu9x', 'muc', 'mu9c', 'muo', 'mu9f', 'dn', 'nbqar', 'nbtbr', 'nbtnr', 'nntnr', 'nbqcr', 'nbqer', 'nbear', 'nbevr', 'nbcer', 'nbitr', 'nbmar', 'nbmnr', 'nbmcr', 'nbmur', 'nbqnr', 'nncl', 'npupr', 'nban', 'nbah', 'nbbi', 'nbbu', 'nbch', 'nbes', 'nbea', 'nben', 'nbev', 'nbig', 'nbit', 'nblw', 'nbma', 'nbmt', 'nbmu', 'nbdn', 'nbph', 'nbso', 'nbss', 'nddo', 'ndhe', 'ndla', 'ndph', 'ndsh', 'nlxx', 'nrxx', 'nsxx', 'ncmh', 'ncme', 'ncsc', 'nfge', 'nucl', 'nu03u', 'nuht', 'nu01u', 'nu02u', 'nu03b', 'nu01b', 'nu02b', 'nbphr', 'nbtur', 'ndspr', 'nlyrr', 'ncspr', 'nfspr', 'php', 'phs', 'so', 'sos', 'esnb', 'es97', 'eanb', 'eaob', 'ennb', 'nbbir', 'nbchr', 'nbdnr', 'ndag')</t>
         </is>
       </c>
       <c r="B170" s="39" t="inlineStr">
@@ -11540,7 +11540,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="173">
       <c r="A173" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in Executive/Management; Faculty/Academic Staff; GTU Faculty; GTU Staff/Visiting Scholar; Howard Hughes Institute; LBNL Academic Staff; Mathematical Sciences Research Institute; Proxy - Faculty; Stanford Faculty; UC Extension Faculty; UCB Academic Dept Affiliate No Proxy; UCB Post-doc; UCB Visiting Scholar</t>
+          <t>"Borrower Details"."User Group" IN ('Executive/Management', 'Faculty/Academic Staff', 'GTU Faculty', 'GTU Staff/Visiting Scholar', 'Howard Hughes Institute', 'LBNL Academic Staff', 'Mathematical Sciences Research Institute', 'Proxy - Faculty', 'Stanford Faculty', 'UC Extension Faculty', 'UCB Academic Dept Affiliate No Proxy', 'UCB Post-doc', 'UCB Visiting Scholar')</t>
         </is>
       </c>
       <c r="B173" s="39" t="inlineStr">
@@ -11607,7 +11607,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="174">
       <c r="A174" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in Graduate Student; GTU Graduate Student; Stanford Graduate Student</t>
+          <t>"Borrower Details"."User Group" IN ('Graduate Student', 'GTU Graduate Student', 'Stanford Graduate Student')</t>
         </is>
       </c>
       <c r="B174" s="39" t="inlineStr">
@@ -11674,7 +11674,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="175">
       <c r="A175" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in LBNL Guest/Temp/Contractor; LBNL Non-Academic/Post-doc; LBNL Retired Staff; Library Departmental Card; Library Development; Library Retired Staff; Library Staff; LLNL Academic Staff; LLNL Non-Academic Staff/Post-doc; LLNL Retired Staff; Non-Academic Retired Staff; Non-Academic Staff; Other UC Retiree; UC Office of the President</t>
+          <t>"Borrower Details"."User Group" IN ('LBNL Guest/Temp/Contractor', 'LBNL Non-Academic/Post-doc', 'LBNL Retired Staff', 'Library Departmental Card', 'Library Development', 'Library Retired Staff', 'Library Staff', 'LLNL Academic Staff', 'LLNL Non-Academic Staff/Post-doc', 'LLNL Retired Staff', 'Non-Academic Retired Staff', 'Non-Academic Staff', 'Other UC Retiree', 'UC Office of the President')</t>
         </is>
       </c>
       <c r="B175" s="39" t="inlineStr">
@@ -11741,7 +11741,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="176">
       <c r="A176" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in UC Extension Student; UC Extension Student Non-concurrent; Undergraduate; Undergraduate - UCB SLE</t>
+          <t>"Borrower Details"."User Group" IN ('UC Extension Student', 'UC Extension Student Non-concurrent', 'Undergraduate', 'Undergraduate - UCB SLE')</t>
         </is>
       </c>
       <c r="B176" s="39" t="inlineStr">
@@ -11808,7 +11808,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="177">
       <c r="A177" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in Alumni; Alumni Lifetime; Botanical Garden Docent; Faculty/Academic Spouse; Faculty/Academic Staff Children; Institute for Historical Study; Non-Academic Staff Spouse; Reference Use Only; UCB Academic Dept Affiliate; UCB Alumni Association Staff</t>
+          <t>"Borrower Details"."User Group" IN ('Alumni', 'Alumni Lifetime', 'Botanical Garden Docent', 'Faculty/Academic Spouse', 'Faculty/Academic Staff Children', 'Institute for Historical Study', 'Non-Academic Staff Spouse', 'Reference Use Only', 'UCB Academic Dept Affiliate', 'UCB Alumni Association Staff')</t>
         </is>
       </c>
       <c r="B177" s="39" t="inlineStr">
@@ -11875,7 +11875,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="178">
       <c r="A178" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in CA Private Univ/Coll Student; CA Public School Teachers; CA Resident; CA University/Colleges Faculty; CA University/Colleges Student; Library Non-Affiliated Users; Other UC Spouse; CA Private School Teachers; Dept of Health Services (DHS); ICSI_MSRI; Library Volunteer</t>
+          <t>"Borrower Details"."User Group" IN ('CA Private Univ/Coll Student', 'CA Public School Teachers', 'CA Resident', 'CA University/Colleges Faculty', 'CA University/Colleges Student', 'Library Non-Affiliated Users', 'Other UC Spouse', 'CA Private School Teachers', 'Dept of Health Services (DHS)', 'ICSI_MSRI', 'Library Volunteer')</t>
         </is>
       </c>
       <c r="B178" s="39" t="inlineStr">
@@ -11942,7 +11942,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="179">
       <c r="A179" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in NETWORK; Network</t>
+          <t>"Borrower Details"."User Group" IN ('NETWORK', 'Network')</t>
         </is>
       </c>
       <c r="B179" s="39" t="inlineStr">
@@ -12009,7 +12009,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="180">
       <c r="A180" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in ILL Other Libraries; ILL UC</t>
+          <t>"Borrower Details"."User Group" IN ('ILL Other Libraries', 'ILL UC')</t>
         </is>
       </c>
       <c r="B180" s="39" t="inlineStr">
@@ -12076,7 +12076,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="181">
       <c r="A181" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group"</t>
+          <t>"Borrower Details"."User Group" IS NULL</t>
         </is>
       </c>
       <c r="B181" s="39" t="inlineStr">
@@ -12143,7 +12143,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="182">
       <c r="A182" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group" is equal to / is in SLF-N Departmental Card; SLF-N/UCB Google Cart; Test Patron Graduate; Test Patron Undergraduate; NRLF Departmental Card; NRLF/UCB Google Cart</t>
+          <t>"Borrower Details"."User Group" IN ('SLF-N Departmental Card', 'SLF-N/UCB Google Cart', 'Test Patron Graduate', 'Test Patron Undergraduate', 'NRLF Departmental Card', 'NRLF/UCB Google Cart')</t>
         </is>
       </c>
       <c r="B182" s="39" t="inlineStr">
@@ -12210,7 +12210,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="183">
       <c r="A183" s="32" t="inlineStr">
         <is>
-          <t>"Borrower Details"."User Group"UC Visiting Scholar/Post-doc</t>
+          <t>"Borrower Details"."User Group" = 'UC Visiting Scholar/Post-doc'</t>
         </is>
       </c>
       <c r="B183" s="39" t="inlineStr">
@@ -12612,7 +12612,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="189">
       <c r="A189" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in zw</t>
+          <t>"Location"."Location Code" LIKE '%zw'</t>
         </is>
       </c>
       <c r="B189" s="39" t="inlineStr">
@@ -13081,7 +13081,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="196">
       <c r="A196" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ah; ah9t; dl; dn; dr; gs; ma9x; mf; mo; ss</t>
+          <t>("Location"."Location Code" LIKE 'ah%' OR "Location"."Location Code" LIKE 'ah9t%' OR "Location"."Location Code" LIKE 'dl%' OR "Location"."Location Code" LIKE 'dn%' OR "Location"."Location Code" LIKE 'dr%' OR "Location"."Location Code" LIKE 'gs%' OR "Location"."Location Code" LIKE 'ma9x%' OR "Location"."Location Code" LIKE 'mf%' OR "Location"."Location Code" LIKE 'mo%' OR "Location"."Location Code" LIKE 'ss%')</t>
         </is>
       </c>
       <c r="B196" s="39" t="inlineStr">
@@ -13148,7 +13148,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="197">
       <c r="A197" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in tb; tj</t>
+          <t>("Location"."Location Code" LIKE 'tb%' OR "Location"."Location Code" LIKE 'tj%')</t>
         </is>
       </c>
       <c r="B197" s="39" t="inlineStr">
@@ -13282,7 +13282,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="199">
       <c r="A199" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in mt</t>
+          <t>"Location"."Location Code" LIKE 'mt%'</t>
         </is>
       </c>
       <c r="B199" s="39" t="inlineStr">
@@ -13349,7 +13349,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="200">
       <c r="A200" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ma</t>
+          <t>"Location"."Location Code" LIKE 'ma%'</t>
         </is>
       </c>
       <c r="B200" s="39" t="inlineStr">
@@ -13416,7 +13416,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="201">
       <c r="A201" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in bu</t>
+          <t>"Location"."Location Code" LIKE 'bu%'</t>
         </is>
       </c>
       <c r="B201" s="39" t="inlineStr">
@@ -13483,7 +13483,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="202">
       <c r="A202" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in mu</t>
+          <t>"Location"."Location Code" LIKE 'mu%'</t>
         </is>
       </c>
       <c r="B202" s="39" t="inlineStr">
@@ -13550,7 +13550,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="203">
       <c r="A203" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in so</t>
+          <t>"Location"."Location Code" LIKE 'so%'</t>
         </is>
       </c>
       <c r="B203" s="39" t="inlineStr">
@@ -13617,7 +13617,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="204">
       <c r="A204" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ch</t>
+          <t>"Location"."Location Code" LIKE 'ch%'</t>
         </is>
       </c>
       <c r="B204" s="39" t="inlineStr">
@@ -13684,7 +13684,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="205">
       <c r="A205" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in an</t>
+          <t>"Location"."Location Code" LIKE 'an%'</t>
         </is>
       </c>
       <c r="B205" s="39" t="inlineStr">
@@ -13751,7 +13751,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="206">
       <c r="A206" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in es</t>
+          <t>"Location"."Location Code" LIKE 'es%'</t>
         </is>
       </c>
       <c r="B206" s="39" t="inlineStr">
@@ -13818,7 +13818,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="207">
       <c r="A207" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in it</t>
+          <t>"Location"."Location Code" LIKE 'it%'</t>
         </is>
       </c>
       <c r="B207" s="39" t="inlineStr">
@@ -13885,7 +13885,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="208">
       <c r="A208" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code"ite</t>
+          <t>"Location"."Location Code" = 'ite'</t>
         </is>
       </c>
       <c r="B208" s="39" t="inlineStr">
@@ -13952,7 +13952,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="209">
       <c r="A209" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in oh</t>
+          <t>"Location"."Location Code" LIKE 'oh%'</t>
         </is>
       </c>
       <c r="B209" s="39" t="inlineStr">
@@ -14019,7 +14019,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="210">
       <c r="A210" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in mc</t>
+          <t>"Location"."Location Code" LIKE 'mc%'</t>
         </is>
       </c>
       <c r="B210" s="39" t="inlineStr">
@@ -14086,7 +14086,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="211">
       <c r="A211" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ig</t>
+          <t>"Location"."Location Code" LIKE 'ig%'</t>
         </is>
       </c>
       <c r="B211" s="39" t="inlineStr">
@@ -14153,7 +14153,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="212">
       <c r="A212" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in qax; qcx; qnx</t>
+          <t>"Location"."Location Code" IN ('qax', 'qcx', 'qnx')</t>
         </is>
       </c>
       <c r="B212" s="39" t="inlineStr">
@@ -14220,7 +14220,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="213">
       <c r="A213" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in lawb; wb</t>
+          <t>"Location"."Location Code" IN ('lawb', 'wb')</t>
         </is>
       </c>
       <c r="B213" s="39" t="inlineStr">
@@ -14287,7 +14287,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="214">
       <c r="A214" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ph</t>
+          <t>"Location"."Location Code" LIKE 'ph%'</t>
         </is>
       </c>
       <c r="B214" s="39" t="inlineStr">
@@ -14354,7 +14354,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="215">
       <c r="A215" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in n</t>
+          <t>"Location"."Location Code" LIKE 'n%'</t>
         </is>
       </c>
       <c r="B215" s="39" t="inlineStr">
@@ -14421,7 +14421,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="216">
       <c r="A216" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in bi</t>
+          <t>"Location"."Location Code" LIKE 'bi%'</t>
         </is>
       </c>
       <c r="B216" s="39" t="inlineStr">
@@ -14488,7 +14488,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="217">
       <c r="A217" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in ev; ce</t>
+          <t>("Location"."Location Code" LIKE 'ev%' OR "Location"."Location Code" LIKE 'ce%')</t>
         </is>
       </c>
       <c r="B217" s="39" t="inlineStr">
@@ -14555,7 +14555,7 @@
     <row collapsed="0" hidden="0" outlineLevel="5" r="218">
       <c r="A218" s="32" t="inlineStr">
         <is>
-          <t>"Location"."Location Code" is equal to / is in qa; qc; qe; qn</t>
+          <t>("Location"."Location Code" LIKE 'qa%' OR "Location"."Location Code" LIKE 'qc%' OR "Location"."Location Code" LIKE 'qe%' OR "Location"."Location Code" LIKE 'qn%')</t>
         </is>
       </c>
       <c r="B218" s="39" t="inlineStr">

</xml_diff>